<commit_message>
feat(serialization): introduce multi-range support in serialization tests
- Added a new script `generate_serialization_spreadsheet.py` to create XLSX files for testing multi-range `=PYTHON()` functionality.
- Updated existing serialization cases to include multi-range scenarios, enhancing the test coverage for the `=PYTHON()` function.
- Modified documentation to reflect changes in serialization test structure and the introduction of multi-range capabilities.
- Adjusted related tests to ensure proper handling of multi-range inputs and outputs in the serialization framework.
</commit_message>
<xml_diff>
--- a/tests/fixtures/serialization_tests.xlsx
+++ b/tests/fixtures/serialization_tests.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="147">
   <si>
     <t xml:space="preserve">test_id</t>
   </si>
@@ -76,7 +76,7 @@
     <t xml:space="preserve">notes</t>
   </si>
   <si>
-    <t xml:space="preserve">python_formula</t>
+    <t xml:space="preserve">PYTHON_formula</t>
   </si>
   <si>
     <t xml:space="preserve">[normal]</t>
@@ -169,18 +169,6 @@
     <t xml:space="preserve">10 cells: first size that uses split_grid (BINARY_MIN_CELLS). SUM 1..10 = 55.</t>
   </si>
   <si>
-    <t xml:space="preserve">row_10_sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1×10 row SUM — split_grid flat 1D shape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">split_grid,flat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10-cell row: split_grid with 1D shape on wire. SUM 1..10 = 55.</t>
-  </si>
-  <si>
     <t xml:space="preserve">grid_4x4_sum</t>
   </si>
   <si>
@@ -235,7 +223,7 @@
     <t xml:space="preserve">1.0</t>
   </si>
   <si>
-    <t xml:space="preserve">Manual CSV uses 1/0 (Calc logical SUM semantics; CSV import does not run =TRUE()).</t>
+    <t xml:space="preserve">Manual sheet uses 1/0 (Calc logical SUM semantics; import does not run =TRUE()).</t>
   </si>
   <si>
     <t xml:space="preserve">bool_false</t>
@@ -247,7 +235,7 @@
     <t xml:space="preserve">0.0</t>
   </si>
   <si>
-    <t xml:space="preserve">Manual CSV uses 1/0 (Calc logical SUM semantics; CSV import does not run =FALSE()).</t>
+    <t xml:space="preserve">Manual sheet uses 1/0 (Calc logical SUM semantics; import does not run =FALSE()).</t>
   </si>
   <si>
     <t xml:space="preserve">bool_col_11_sum</t>
@@ -262,7 +250,7 @@
     <t xml:space="preserve">7.0</t>
   </si>
   <si>
-    <t xml:space="preserve">11 cells forces split_grid; CSV uses 1/0 per cell.</t>
+    <t xml:space="preserve">11 cells forces split_grid; sheet uses 1/0 per cell.</t>
   </si>
   <si>
     <t xml:space="preserve">row_5</t>
@@ -284,6 +272,75 @@
   </si>
   <si>
     <t xml:space="preserve">row_11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[multi]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_two_2x2_sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two 2×2 ranges — combined SUM (1+2+3+4+5+6+7+8=36)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_range,varargs,below_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data[0] and data[1] are 2×2; oracle =SUM(r1,r2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_2x1_plus_1x2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2×1 column + 1×2 row — shape mismatch (1+2+3+4=10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exercises list-of-grids wire (not one 2D block).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_two_rows_sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two 1×3 rows — flat per-range lists (1+2+3+4+5+6=21)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_range,varargs,flat,below_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_scalar_plus_row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Single cell + 1×3 row — scalar range + flat list (5+1+2+3=11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_mixed_small</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed 2×2 + numeric 1×1 — numeric-only sum (1+2+3=6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">multi_range,varargs,mixed,below_threshold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strings in range 1; Calc SUM skips text in oracle cells.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
   </si>
   <si>
     <t xml:space="preserve">[mixed]</t>
@@ -784,7 +841,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R111"/>
+  <dimension ref="A1:R128"/>
   <sheetFormatPr defaultColWidth="8.2265625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -795,7 +852,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1196,22 +1253,22 @@
         <v>50</v>
       </c>
       <c r="N26" s="0" t="n">
-        <f aca="false">SUM(D27:M27)</f>
-        <v>55</v>
+        <f aca="false">SUM(D27:G30)</f>
+        <v>136</v>
       </c>
       <c r="O26" s="0" t="str">
         <f aca="false">IF(ABS(N26-R26)&lt;0.001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P26" s="0" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="Q26" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="R26" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D27:M27)</f>
-        <v>55</v>
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D27:G30)</f>
+        <v>136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1230,317 +1287,290 @@
       <c r="G27" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="H27" s="0" t="n">
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="I27" s="0" t="n">
+      <c r="E28" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="J27" s="0" t="n">
+      <c r="F28" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="K27" s="0" t="n">
+      <c r="G28" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="L27" s="0" t="n">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="M27" s="0" t="n">
+      <c r="E29" s="0" t="n">
         <v>10</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>52</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="N29" s="0" t="n">
-        <f aca="false">SUM(D30:G33)</f>
-        <v>136</v>
-      </c>
-      <c r="O29" s="0" t="str">
-        <f aca="false">IF(ABS(N29-R29)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P29" s="0" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q29" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="R29" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D30:G33)</f>
-        <v>136</v>
+      <c r="F29" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="G29" s="0" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D30" s="0" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E30" s="0" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F30" s="0" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G30" s="0" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="E31" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="F31" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="G31" s="0" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D32" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E32" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="F32" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G32" s="0" t="n">
-        <v>12</v>
+        <v>53</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="N32" s="0" t="n">
+        <f aca="false">SUM(D33:F36)</f>
+        <v>78</v>
+      </c>
+      <c r="O32" s="0" t="str">
+        <f aca="false">IF(ABS(N32-R32)&lt;0.001,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P32" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q32" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="R32" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D33:F36)</f>
+        <v>78</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D33" s="0" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E33" s="0" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="F33" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="G33" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>57</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C35" s="0" t="s">
-        <v>59</v>
-      </c>
-      <c r="N35" s="0" t="n">
-        <f aca="false">SUM(D36:F39)</f>
-        <v>78</v>
-      </c>
-      <c r="O35" s="0" t="str">
-        <f aca="false">IF(ABS(N35-R35)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P35" s="0" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q35" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="R35" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D36:F39)</f>
-        <v>78</v>
+        <v>32</v>
+      </c>
+      <c r="D35" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="F35" s="0" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D36" s="0" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E36" s="0" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F36" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D37" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="E37" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="F37" s="0" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D38" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="E38" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="F38" s="0" t="n">
-        <v>9</v>
+        <v>58</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="N38" s="0" t="n">
+        <f aca="false">MAX(D39:G42)</f>
+        <v>16</v>
+      </c>
+      <c r="O38" s="0" t="str">
+        <f aca="false">IF(ABS(N38-R38)&lt;0.001,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P38" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q38" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="R38" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.max(data)",D39:G42)</f>
+        <v>16</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D39" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G39" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G40" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="E39" s="0" t="n">
+      <c r="F41" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="F39" s="0" t="n">
+      <c r="G41" s="0" t="n">
         <v>12</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>62</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C41" s="0" t="s">
-        <v>54</v>
-      </c>
-      <c r="N41" s="0" t="n">
-        <f aca="false">MAX(D42:G45)</f>
-        <v>16</v>
-      </c>
-      <c r="O41" s="0" t="str">
-        <f aca="false">IF(ABS(N41-R41)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P41" s="0" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q41" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="R41" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.max(data)",D42:G45)</f>
-        <v>16</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D42" s="0" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E42" s="0" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F42" s="0" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G42" s="0" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D43" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="E43" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="F43" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="G43" s="0" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="42.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D44" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E44" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="F44" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G44" s="0" t="n">
-        <v>12</v>
+        <v>62</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="N44" s="0" t="n">
+        <f aca="false">SUM(D45)</f>
+        <v>1</v>
+      </c>
+      <c r="O44" s="0" t="str">
+        <f aca="false">IF(ABS(N44-R44)&lt;0.001,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P44" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q44" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="R44" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D45)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D45" s="0" t="n">
-        <v>13</v>
-      </c>
-      <c r="E45" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="F45" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="G45" s="0" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="42.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="N47" s="0" t="n">
         <f aca="false">SUM(D48)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O47" s="0" t="str">
         <f aca="false">IF(ABS(N47-R47)&lt;0.001,"PASS","FAIL")</f>
@@ -1554,7 +1584,7 @@
       </c>
       <c r="R47" s="4" t="n">
         <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D48)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1562,10 +1592,10 @@
         <v>27</v>
       </c>
       <c r="D48" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="42.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
         <v>71</v>
       </c>
@@ -1573,25 +1603,25 @@
         <v>72</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="N50" s="0" t="n">
-        <f aca="false">SUM(D51)</f>
-        <v>0</v>
+        <f aca="false">SUM(D51:D61)</f>
+        <v>7</v>
       </c>
       <c r="O50" s="0" t="str">
         <f aca="false">IF(ABS(N50-R50)&lt;0.001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
       <c r="P50" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="Q50" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R50" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D51)</f>
-        <v>0</v>
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D51:D61)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1599,49 +1629,36 @@
         <v>27</v>
       </c>
       <c r="D51" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D52" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>75</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C53" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N53" s="0" t="n">
-        <f aca="false">SUM(D54:D64)</f>
-        <v>7</v>
-      </c>
-      <c r="O53" s="0" t="str">
-        <f aca="false">IF(ABS(N53-R53)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P53" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="Q53" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="R53" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.sum(data)",D54:D64)</f>
-        <v>7</v>
+        <v>32</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D54" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>31</v>
+        <v>76</v>
       </c>
       <c r="D55" s="0" t="n">
         <v>1</v>
@@ -1649,39 +1666,39 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>32</v>
+        <v>77</v>
       </c>
       <c r="D56" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="D57" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D58" s="0" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D59" s="0" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D60" s="0" t="n">
         <v>1</v>
@@ -1689,251 +1706,292 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="0" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D61" s="0" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="0" t="s">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+      <c r="L64" s="3"/>
+      <c r="M64" s="3"/>
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
+      <c r="P64" s="3"/>
+      <c r="Q64" s="3"/>
+      <c r="R64" s="3"/>
+    </row>
+    <row r="65" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="D62" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
+      <c r="B65" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="D63" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
+      <c r="C65" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="D64" s="0" t="n">
-        <v>0</v>
+      <c r="N65" s="0" t="n">
+        <f aca="false">SUM(D66:E67,I66:J67)</f>
+        <v>36</v>
+      </c>
+      <c r="O65" s="0" t="e">
+        <f aca="false">IF(ABS(N65-R65)&lt;0.001,"PASS","FAIL")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P65" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q65" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="R65" s="4" t="e">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(np.sum(d) for d in data)",D66:E67,I66:J67)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="I66" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J66" s="0" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="3"/>
-      <c r="I67" s="3"/>
-      <c r="J67" s="3"/>
-      <c r="K67" s="3"/>
-      <c r="L67" s="3"/>
-      <c r="M67" s="3"/>
-      <c r="N67" s="3"/>
-      <c r="O67" s="3"/>
-      <c r="P67" s="3"/>
-      <c r="Q67" s="3"/>
-      <c r="R67" s="3"/>
-    </row>
-    <row r="68" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="B68" s="4" t="s">
+      <c r="A67" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D67" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E67" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="I67" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="J67" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="C68" s="0" t="s">
+      <c r="B69" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="N68" s="0" t="str">
-        <f aca="false">INDEX(D69:F69,1)</f>
-        <v>02138</v>
-      </c>
-      <c r="O68" s="0" t="str">
-        <f aca="false">IF(R68="02138","PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P68" s="0" t="s">
+      <c r="C69" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="N69" s="0" t="n">
+        <f aca="false">SUM(D70:D71,I70:J70)</f>
+        <v>10</v>
+      </c>
+      <c r="O69" s="0" t="e">
+        <f aca="false">IF(ABS(N69-R69)&lt;0.001,"PASS","FAIL")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P69" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q69" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="Q68" s="4" t="s">
+      <c r="R69" s="4" t="e">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(np.sum(d) for d in data)",D70:D71,I70:J70)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="I70" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="J70" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D71" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="R68" s="4" t="str">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data[0]",D69:F69)</f>
-        <v>02138</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="D69" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="E69" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="0" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="0" t="s">
+      <c r="B73" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="B71" s="4" t="s">
+      <c r="C73" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="C71" s="0" t="s">
+      <c r="N73" s="0" t="n">
+        <f aca="false">SUM(D74:F74,I74:K74)</f>
+        <v>21</v>
+      </c>
+      <c r="O73" s="0" t="e">
+        <f aca="false">IF(ABS(N73-R73)&lt;0.001,"PASS","FAIL")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P73" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="N71" s="0" t="n">
-        <f aca="false">SUM(D72:F75)</f>
-        <v>110</v>
-      </c>
-      <c r="O71" s="0" t="str">
-        <f aca="false">IF(ABS(N71-R71)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P71" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q71" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="R71" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(v for row in data for v in row if isinstance(v, (int, float)))",D72:F75)</f>
-        <v>110</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="D72" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="F72" s="0" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D73" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="F73" s="0" t="n">
-        <v>20</v>
+      <c r="R73" s="4" t="e">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(np.sum(d) for d in data)",D74:F74,I74:K74)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="0" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D74" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="E74" s="0" t="s">
+      <c r="I74" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="J74" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="K74" s="0" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C76" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="N76" s="0" t="n">
+        <f aca="false">SUM(D77,I77:K77)</f>
+        <v>11</v>
+      </c>
+      <c r="O76" s="0" t="e">
+        <f aca="false">IF(ABS(N76-R76)&lt;0.001,"PASS","FAIL")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P76" s="0" t="s">
+        <v>98</v>
+      </c>
+      <c r="R76" s="4" t="e">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(np.sum(d) for d in data)",D77,I77:K77)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D77" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="I77" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J77" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="F74" s="0" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D75" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="E75" s="0" t="s">
+      <c r="B79" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F75" s="0" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="0" t="s">
+      <c r="C79" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="B77" s="4" t="s">
+      <c r="N79" s="0" t="n">
+        <f aca="false">SUM(D80:E81,I80)</f>
+        <v>6</v>
+      </c>
+      <c r="O79" s="0" t="e">
+        <f aca="false">IF(ABS(N79-R79)&lt;0.001,"PASS","FAIL")</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="P79" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="C77" s="0" t="s">
+      <c r="Q79" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="N77" s="0" t="str">
-        <f aca="false">INDEX(D78:E81,1,1)</f>
-        <v>São Paulo</v>
-      </c>
-      <c r="O77" s="0" t="str">
-        <f aca="false">IF(R77="São Paulo","PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P77" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="R77" s="4" t="str">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data[0]",D78:E81)</f>
-        <v>São Paulo</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="D78" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="E78" s="0" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="E79" s="0" t="n">
-        <v>7</v>
+      <c r="R79" s="4" t="e">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(v for g in data for row in g for v in row if isinstance(v, (int, float)))",D80:E81,I80)</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="E80" s="0" t="n">
-        <v>9</v>
+        <v>27</v>
+      </c>
+      <c r="D80" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="I80" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="0" t="s">
-        <v>33</v>
-      </c>
-      <c r="D81" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="E81" s="0" t="n">
-        <v>11</v>
+        <v>31</v>
+      </c>
+      <c r="D81" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E81" s="0" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1968,383 +2026,601 @@
       <c r="C85" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="N85" s="0" t="e">
-        <f aca="false">INDEX(D86:G89,ROW()-85,COLUMN()-3)*2</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O85" s="0" t="s">
+      <c r="N85" s="0" t="str">
+        <f aca="false">INDEX(D86:F86,1)</f>
+        <v>02138</v>
+      </c>
+      <c r="O85" s="0" t="str">
+        <f aca="false">IF(R85="02138","PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P85" s="0" t="s">
         <v>110</v>
       </c>
       <c r="Q85" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="R85" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.array(data) * 2",D86:G89)</f>
-        <v>2</v>
+      <c r="R85" s="4" t="str">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data[0]",D86:F86)</f>
+        <v>02138</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="D86" s="0" t="n">
-        <v>1</v>
+      <c r="D86" s="0" t="s">
+        <v>110</v>
       </c>
       <c r="E86" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="F86" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G86" s="0" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D87" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="E87" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="F87" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="G87" s="0" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="88" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D88" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E88" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="F88" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G88" s="0" t="n">
-        <v>12</v>
+        <v>112</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C88" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="N88" s="0" t="n">
+        <f aca="false">SUM(D89:F92)</f>
+        <v>110</v>
+      </c>
+      <c r="O88" s="0" t="str">
+        <f aca="false">IF(ABS(N88-R88)&lt;0.001,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P88" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q88" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="R88" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("sum(v for row in data for v in row if isinstance(v, (int, float)))",D89:F92)</f>
+        <v>110</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="0" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D89" s="0" t="n">
-        <v>13</v>
-      </c>
-      <c r="E89" s="0" t="n">
-        <v>14</v>
+        <v>1</v>
+      </c>
+      <c r="E89" s="0" t="s">
+        <v>116</v>
       </c>
       <c r="F89" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="G89" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E90" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="F90" s="0" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C91" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="N91" s="0" t="e">
-        <f aca="false">INDEX(D92:G95,ROW()-91,COLUMN()-3)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="O91" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q91" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="R91" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data",D92:G95)</f>
-        <v>1</v>
+        <v>32</v>
+      </c>
+      <c r="D91" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E91" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="F91" s="0" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D92" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E92" s="0" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="E92" s="0" t="s">
+        <v>119</v>
       </c>
       <c r="F92" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G92" s="0" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D93" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="E93" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="F93" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="G93" s="0" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D94" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E94" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="F94" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G94" s="0" t="n">
-        <v>12</v>
+        <v>120</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C94" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="N94" s="0" t="str">
+        <f aca="false">INDEX(D95:E98,1,1)</f>
+        <v>São Paulo</v>
+      </c>
+      <c r="O94" s="0" t="str">
+        <f aca="false">IF(R94="São Paulo","PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P94" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="R94" s="4" t="str">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data[0]",D95:E98)</f>
+        <v>São Paulo</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D95" s="0" t="s">
+        <v>123</v>
+      </c>
+      <c r="E95" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D96" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E96" s="0" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="E97" s="0" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="D95" s="0" t="n">
-        <v>13</v>
-      </c>
-      <c r="E95" s="0" t="n">
-        <v>14</v>
-      </c>
-      <c r="F95" s="0" t="n">
-        <v>15</v>
-      </c>
-      <c r="G95" s="0" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B98" s="3"/>
-      <c r="C98" s="3"/>
-      <c r="D98" s="3"/>
-      <c r="E98" s="3"/>
-      <c r="F98" s="3"/>
-      <c r="G98" s="3"/>
-      <c r="H98" s="3"/>
-      <c r="I98" s="3"/>
-      <c r="J98" s="3"/>
-      <c r="K98" s="3"/>
-      <c r="L98" s="3"/>
-      <c r="M98" s="3"/>
-      <c r="N98" s="3"/>
-      <c r="O98" s="3"/>
-      <c r="P98" s="3"/>
-      <c r="Q98" s="3"/>
-      <c r="R98" s="3"/>
-    </row>
-    <row r="99" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="B99" s="4" t="s">
+      <c r="D98" s="0" t="s">
         <v>117</v>
       </c>
-      <c r="C99" s="0" t="s">
-        <v>118</v>
-      </c>
-      <c r="N99" s="0" t="n">
-        <f aca="false">SUM(D100:G103)</f>
-        <v>114</v>
-      </c>
-      <c r="O99" s="0" t="str">
-        <f aca="false">IF(ABS(N99-R99)&lt;0.001,"PASS","FAIL")</f>
-        <v>PASS</v>
-      </c>
-      <c r="P99" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="Q99" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="R99" s="4" t="n">
-        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.nansum(data)",D100:G103)</f>
-        <v>114</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="D100" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F100" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="G100" s="0" t="n">
-        <v>4</v>
+      <c r="E98" s="0" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="D101" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="E101" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="G101" s="0" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B101" s="3"/>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3"/>
+      <c r="E101" s="3"/>
+      <c r="F101" s="3"/>
+      <c r="G101" s="3"/>
+      <c r="H101" s="3"/>
+      <c r="I101" s="3"/>
+      <c r="J101" s="3"/>
+      <c r="K101" s="3"/>
+      <c r="L101" s="3"/>
+      <c r="M101" s="3"/>
+      <c r="N101" s="3"/>
+      <c r="O101" s="3"/>
+      <c r="P101" s="3"/>
+      <c r="Q101" s="3"/>
+      <c r="R101" s="3"/>
+    </row>
+    <row r="102" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D102" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="E102" s="0" t="n">
-        <v>10</v>
-      </c>
-      <c r="F102" s="0" t="n">
-        <v>11</v>
-      </c>
-      <c r="G102" s="0" t="n">
-        <v>12</v>
+        <v>126</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C102" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="N102" s="0" t="e">
+        <f aca="false">INDEX(D103:G106,ROW()-102,COLUMN()-3)*2</f>
+        <v>#REF!</v>
+      </c>
+      <c r="O102" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q102" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="R102" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.array(data) * 2",D103:G106)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D103" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G103" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D104" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E104" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="F104" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G104" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D105" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="E105" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="F105" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="G105" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="0" t="s">
         <v>33</v>
       </c>
-      <c r="E103" s="0" t="n">
+      <c r="D106" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="E106" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="F103" s="0" t="n">
+      <c r="F106" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="G103" s="0" t="n">
+      <c r="G106" s="0" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="B106" s="3"/>
-      <c r="C106" s="3"/>
-      <c r="D106" s="3"/>
-      <c r="E106" s="3"/>
-      <c r="F106" s="3"/>
-      <c r="G106" s="3"/>
-      <c r="H106" s="3"/>
-      <c r="I106" s="3"/>
-      <c r="J106" s="3"/>
-      <c r="K106" s="3"/>
-      <c r="L106" s="3"/>
-      <c r="M106" s="3"/>
-      <c r="N106" s="3"/>
-      <c r="O106" s="3"/>
-      <c r="P106" s="3"/>
-      <c r="Q106" s="3"/>
-      <c r="R106" s="3"/>
-    </row>
-    <row r="107" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0" t="s">
-        <v>122</v>
-      </c>
-      <c r="B107" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C107" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="O107" s="0" t="str">
-        <f aca="false">IF(LEFT(R107,6)="Error:","PASS","FAIL")</f>
+    <row r="108" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="0" t="s">
+        <v>131</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C108" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="N108" s="0" t="e">
+        <f aca="false">INDEX(D109:G112,ROW()-108,COLUMN()-3)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="O108" s="0" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q108" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="R108" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("data",D109:G112)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D109" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="F109" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G109" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D110" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E110" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="F110" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="G110" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D111" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="E111" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="F111" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="G111" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="D112" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="E112" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="F112" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="G112" s="0" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B115" s="3"/>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3"/>
+      <c r="E115" s="3"/>
+      <c r="F115" s="3"/>
+      <c r="G115" s="3"/>
+      <c r="H115" s="3"/>
+      <c r="I115" s="3"/>
+      <c r="J115" s="3"/>
+      <c r="K115" s="3"/>
+      <c r="L115" s="3"/>
+      <c r="M115" s="3"/>
+      <c r="N115" s="3"/>
+      <c r="O115" s="3"/>
+      <c r="P115" s="3"/>
+      <c r="Q115" s="3"/>
+      <c r="R115" s="3"/>
+    </row>
+    <row r="116" customFormat="false" ht="29" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C116" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="N116" s="0" t="n">
+        <f aca="false">SUM(D117:G120)</f>
+        <v>114</v>
+      </c>
+      <c r="O116" s="0" t="str">
+        <f aca="false">IF(ABS(N116-R116)&lt;0.001,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="P107" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="R107" s="4" t="str">
+      <c r="P116" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="Q116" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="R116" s="4" t="n">
+        <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("np.nansum(data)",D117:G120)</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="D117" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G117" s="0" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="D118" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E118" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="G118" s="0" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="D119" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="E119" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="F119" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="G119" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E120" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="F120" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="G120" s="0" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B123" s="3"/>
+      <c r="C123" s="3"/>
+      <c r="D123" s="3"/>
+      <c r="E123" s="3"/>
+      <c r="F123" s="3"/>
+      <c r="G123" s="3"/>
+      <c r="H123" s="3"/>
+      <c r="I123" s="3"/>
+      <c r="J123" s="3"/>
+      <c r="K123" s="3"/>
+      <c r="L123" s="3"/>
+      <c r="M123" s="3"/>
+      <c r="N123" s="3"/>
+      <c r="O123" s="3"/>
+      <c r="P123" s="3"/>
+      <c r="Q123" s="3"/>
+      <c r="R123" s="3"/>
+    </row>
+    <row r="124" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C124" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="O124" s="0" t="str">
+        <f aca="false">IF(LEFT(R124,6)="Error:","PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+      <c r="P124" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="R124" s="4" t="str">
         <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("1 +")</f>
         <v>Error: Code parsing failed on line 5 due to: SyntaxError: invalid syntax (&lt;unknown&gt;, line 5)
 1 +
     ^</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0" t="s">
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="D108" s="0" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="110" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0" t="s">
-        <v>126</v>
-      </c>
-      <c r="B110" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C110" s="0" t="s">
-        <v>124</v>
-      </c>
-      <c r="O110" s="0" t="str">
-        <f aca="false">IF(LEFT(R110,6)="Error:","PASS","FAIL")</f>
+      <c r="D125" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="0" t="s">
+        <v>145</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C127" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="O127" s="0" t="str">
+        <f aca="false">IF(LEFT(R127,6)="Error:","PASS","FAIL")</f>
         <v>PASS</v>
       </c>
-      <c r="P110" s="0" t="s">
-        <v>125</v>
-      </c>
-      <c r="R110" s="4" t="str">
+      <c r="P127" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="R127" s="4" t="str">
         <f aca="false">ORG.EXTENSION.WRITERAGENT.PYTHONFUNCTION.PYTHON("import os")</f>
-        <v>Error: Code execution failed at line 'import os' due to: InterpreterError: Import of os is not allowed. Authorized imports are: ['fractions', 'random', 'pandas.*', 'functools', 'scipy', 'statsmodels', 'statsmodels.*', 'seaborn', 'pandas', 'decimal', 'json', 'matplotlib', 'datetime', 'cv2', 'copy', 'scipy.*', 'sympy', 'numpy', 'networkx.*', 'unicodedata', 'dataclasses', 'sklearn.*', 'sklearn', 'numpy.*', 'seaborn.*', 'time', 'csv', 'typing', 'itertools', 'PIL.*', 'statistics', 'textwrap', 'collections', 'platform', 'pprint', 'PIL', 'queue', 'stat', 're', 'enum', 'operator', 'string', 'networkx', 'matplotlib.*', 'math', 'sympy.*']</v>
-      </c>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0" t="s">
+        <v>Error: Code execution failed at line 'import os' due to: InterpreterError: Import of os is not allowed. Authorized imports are: ['enum', 'pandas', 'matplotlib.*', 'textwrap', 'typing', 'cv2', 'math', 'sklearn', 'scipy', 'matplotlib', 'PIL', 'random', 'fractions', 'copy', 'string', 'numpy.*', 'numpy', 'sympy.*', 'itertools', 'statsmodels', 'PIL.*', 'functools', 'json', 'datetime', 're', 'seaborn', 'queue', 'scipy.*', 'statsmodels.*', 'sklearn.*', 'seaborn.*', 'unicodedata', 'sympy', 'collections', 'networkx', 'decimal', 'dataclasses', 'stat', 'time', 'pprint', 'pandas.*', 'statistics', 'operator', 'networkx.*', 'platform', 'csv']</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="0" t="s">
         <v>27</v>
       </c>
-      <c r="D111" s="0" t="n">
+      <c r="D128" s="0" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A67:R67"/>
+    <mergeCell ref="A64:R64"/>
     <mergeCell ref="A84:R84"/>
-    <mergeCell ref="A98:R98"/>
-    <mergeCell ref="A106:R106"/>
+    <mergeCell ref="A101:R101"/>
+    <mergeCell ref="A115:R115"/>
+    <mergeCell ref="A123:R123"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>